<commit_message>
Refactor staff and course management features
- Improved global search functionality in staff and course lists to enhance user experience.
- Added clear button to creatable select inputs for better usability.
- Updated course and staff templates to include total count elements for dynamic updates.
- Enhanced dropdown positioning and visibility for better interaction.
- Modified modal forms for improved layout and user guidance.
- General code cleanup and optimization for maintainability.
</commit_message>
<xml_diff>
--- a/data/Course Data.xlsx
+++ b/data/Course Data.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jainul\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\QPS\qps_paper_settings\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D111E83-3A9A-401E-8FAF-B9CCD71BE21B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67246A66-DC82-406C-94E7-425177448499}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="229" uniqueCount="117">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="228" uniqueCount="116">
   <si>
     <t>Program Type</t>
   </si>
@@ -32,9 +32,6 @@
   </si>
   <si>
     <t>Branch Final</t>
-  </si>
-  <si>
-    <t>ID</t>
   </si>
   <si>
     <t>Course Category</t>
@@ -728,31 +725,30 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:S16"/>
+  <dimension ref="A1:R16"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="12.77734375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="7.109375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="20.77734375" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="11.21875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="3" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="14.88671875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11.5546875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="9" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="28.33203125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="8.77734375" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="4.44140625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="5.88671875" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="6" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="12.44140625" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.6640625" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="10.109375" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="13.44140625" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="14.33203125" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="32.6640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.88671875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.5546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="28.33203125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="8.77734375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="4.44140625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="5.88671875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="6" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="12.44140625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="12.6640625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="10.109375" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="13.44140625" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="14.33203125" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="32.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -807,25 +803,22 @@
       <c r="R1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="1" t="s">
+    </row>
+    <row r="2" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A2" s="2" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="2" spans="1:19" x14ac:dyDescent="0.3">
-      <c r="A2" s="2" t="s">
+      <c r="B2" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="C2" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="D2" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="E2" s="2" t="s">
         <v>22</v>
-      </c>
-      <c r="E2" s="2">
-        <v>1</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>23</v>
@@ -840,25 +833,25 @@
         <v>26</v>
       </c>
       <c r="J2" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="K2" s="2">
+        <v>4</v>
+      </c>
+      <c r="L2" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="K2" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="L2" s="2">
-        <v>4</v>
-      </c>
-      <c r="M2" s="2" t="s">
+      <c r="M2" s="2">
+        <v>40</v>
+      </c>
+      <c r="N2" s="2">
+        <v>60</v>
+      </c>
+      <c r="O2" s="2">
+        <v>100</v>
+      </c>
+      <c r="P2" s="2" t="s">
         <v>28</v>
-      </c>
-      <c r="N2" s="2">
-        <v>40</v>
-      </c>
-      <c r="O2" s="2">
-        <v>60</v>
-      </c>
-      <c r="P2" s="2">
-        <v>100</v>
       </c>
       <c r="Q2" s="2" t="s">
         <v>29</v>
@@ -866,28 +859,25 @@
       <c r="R2" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="S2" s="2" t="s">
+    </row>
+    <row r="3" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A3" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="F3" s="2" t="s">
         <v>31</v>
-      </c>
-    </row>
-    <row r="3" spans="1:19" x14ac:dyDescent="0.3">
-      <c r="A3" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="E3" s="2">
-        <v>2</v>
-      </c>
-      <c r="F3" s="2" t="s">
-        <v>23</v>
       </c>
       <c r="G3" s="2" t="s">
         <v>32</v>
@@ -899,25 +889,25 @@
         <v>34</v>
       </c>
       <c r="J3" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="K3" s="2">
+        <v>5</v>
+      </c>
+      <c r="L3" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="K3" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="L3" s="2">
-        <v>5</v>
-      </c>
-      <c r="M3" s="2" t="s">
+      <c r="M3" s="2">
+        <v>40</v>
+      </c>
+      <c r="N3" s="2">
+        <v>60</v>
+      </c>
+      <c r="O3" s="2">
+        <v>100</v>
+      </c>
+      <c r="P3" s="2" t="s">
         <v>36</v>
-      </c>
-      <c r="N3" s="2">
-        <v>40</v>
-      </c>
-      <c r="O3" s="2">
-        <v>60</v>
-      </c>
-      <c r="P3" s="2">
-        <v>100</v>
       </c>
       <c r="Q3" s="2" t="s">
         <v>37</v>
@@ -925,25 +915,22 @@
       <c r="R3" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="S3" s="2" t="s">
+    </row>
+    <row r="4" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A4" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D4" s="2" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="4" spans="1:19" x14ac:dyDescent="0.3">
-      <c r="A4" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="D4" s="2" t="s">
+      <c r="E4" s="2" t="s">
         <v>40</v>
-      </c>
-      <c r="E4" s="2">
-        <v>3</v>
       </c>
       <c r="F4" s="2" t="s">
         <v>41</v>
@@ -958,54 +945,51 @@
         <v>44</v>
       </c>
       <c r="J4" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="K4" s="2">
+        <v>4</v>
+      </c>
+      <c r="L4" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="M4" s="2">
+        <v>30</v>
+      </c>
+      <c r="N4" s="2">
+        <v>70</v>
+      </c>
+      <c r="O4" s="2">
+        <v>100</v>
+      </c>
+      <c r="P4" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="Q4" s="2" t="s">
         <v>45</v>
-      </c>
-      <c r="K4" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="L4" s="2">
-        <v>4</v>
-      </c>
-      <c r="M4" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="N4" s="2">
-        <v>30</v>
-      </c>
-      <c r="O4" s="2">
-        <v>70</v>
-      </c>
-      <c r="P4" s="2">
-        <v>100</v>
-      </c>
-      <c r="Q4" s="2" t="s">
-        <v>37</v>
       </c>
       <c r="R4" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="S4" s="2" t="s">
+    </row>
+    <row r="5" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A5" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C5" s="2" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="5" spans="1:19" x14ac:dyDescent="0.3">
-      <c r="A5" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="C5" s="2" t="s">
+      <c r="D5" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="D5" s="2" t="s">
+      <c r="E5" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="F5" s="2" t="s">
         <v>49</v>
-      </c>
-      <c r="E5" s="2">
-        <v>4</v>
-      </c>
-      <c r="F5" s="2" t="s">
-        <v>23</v>
       </c>
       <c r="G5" s="2" t="s">
         <v>50</v>
@@ -1014,57 +998,54 @@
         <v>51</v>
       </c>
       <c r="I5" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="J5" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="K5" s="2">
+        <v>4</v>
+      </c>
+      <c r="L5" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="M5" s="2">
+        <v>40</v>
+      </c>
+      <c r="N5" s="2">
+        <v>60</v>
+      </c>
+      <c r="O5" s="2">
+        <v>100</v>
+      </c>
+      <c r="P5" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="Q5" s="2" t="s">
         <v>52</v>
-      </c>
-      <c r="J5" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="K5" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="L5" s="2">
-        <v>4</v>
-      </c>
-      <c r="M5" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="N5" s="2">
-        <v>40</v>
-      </c>
-      <c r="O5" s="2">
-        <v>60</v>
-      </c>
-      <c r="P5" s="2">
-        <v>100</v>
-      </c>
-      <c r="Q5" s="2" t="s">
-        <v>29</v>
       </c>
       <c r="R5" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="S5" s="2" t="s">
+    </row>
+    <row r="6" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A6" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="F6" s="2" t="s">
         <v>54</v>
-      </c>
-    </row>
-    <row r="6" spans="1:19" x14ac:dyDescent="0.3">
-      <c r="A6" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="E6" s="2">
-        <v>5</v>
-      </c>
-      <c r="F6" s="2" t="s">
-        <v>23</v>
       </c>
       <c r="G6" s="2" t="s">
         <v>55</v>
@@ -1073,57 +1054,54 @@
         <v>56</v>
       </c>
       <c r="I6" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="J6" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="K6" s="2">
+        <v>4</v>
+      </c>
+      <c r="L6" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="M6" s="2">
+        <v>35</v>
+      </c>
+      <c r="N6" s="2">
+        <v>65</v>
+      </c>
+      <c r="O6" s="2">
+        <v>100</v>
+      </c>
+      <c r="P6" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="Q6" s="2" t="s">
         <v>57</v>
-      </c>
-      <c r="J6" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="K6" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="L6" s="2">
-        <v>4</v>
-      </c>
-      <c r="M6" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="N6" s="2">
-        <v>35</v>
-      </c>
-      <c r="O6" s="2">
-        <v>65</v>
-      </c>
-      <c r="P6" s="2">
-        <v>100</v>
-      </c>
-      <c r="Q6" s="2" t="s">
-        <v>37</v>
       </c>
       <c r="R6" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="S6" s="2" t="s">
+    </row>
+    <row r="7" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A7" s="2" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="7" spans="1:19" x14ac:dyDescent="0.3">
-      <c r="A7" s="2" t="s">
+      <c r="B7" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="C7" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="F7" s="2" t="s">
         <v>61</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="E7" s="2">
-        <v>6</v>
-      </c>
-      <c r="F7" s="2" t="s">
-        <v>23</v>
       </c>
       <c r="G7" s="2" t="s">
         <v>62</v>
@@ -1132,57 +1110,54 @@
         <v>63</v>
       </c>
       <c r="I7" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="J7" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="K7" s="2">
+        <v>4</v>
+      </c>
+      <c r="L7" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="M7" s="2">
+        <v>40</v>
+      </c>
+      <c r="N7" s="2">
+        <v>60</v>
+      </c>
+      <c r="O7" s="2">
+        <v>100</v>
+      </c>
+      <c r="P7" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="Q7" s="2" t="s">
         <v>64</v>
-      </c>
-      <c r="J7" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="K7" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="L7" s="2">
-        <v>4</v>
-      </c>
-      <c r="M7" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="N7" s="2">
-        <v>40</v>
-      </c>
-      <c r="O7" s="2">
-        <v>60</v>
-      </c>
-      <c r="P7" s="2">
-        <v>100</v>
-      </c>
-      <c r="Q7" s="2" t="s">
-        <v>29</v>
       </c>
       <c r="R7" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="S7" s="2" t="s">
+    </row>
+    <row r="8" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A8" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="F8" s="2" t="s">
         <v>66</v>
-      </c>
-    </row>
-    <row r="8" spans="1:19" x14ac:dyDescent="0.3">
-      <c r="A8" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="E8" s="2">
-        <v>7</v>
-      </c>
-      <c r="F8" s="2" t="s">
-        <v>23</v>
       </c>
       <c r="G8" s="2" t="s">
         <v>67</v>
@@ -1191,175 +1166,166 @@
         <v>68</v>
       </c>
       <c r="I8" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="J8" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="K8" s="2">
+        <v>5</v>
+      </c>
+      <c r="L8" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="M8" s="2">
+        <v>30</v>
+      </c>
+      <c r="N8" s="2">
+        <v>70</v>
+      </c>
+      <c r="O8" s="2">
+        <v>100</v>
+      </c>
+      <c r="P8" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="Q8" s="2" t="s">
         <v>69</v>
-      </c>
-      <c r="J8" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="K8" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="L8" s="2">
-        <v>5</v>
-      </c>
-      <c r="M8" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="N8" s="2">
-        <v>30</v>
-      </c>
-      <c r="O8" s="2">
-        <v>70</v>
-      </c>
-      <c r="P8" s="2">
-        <v>100</v>
-      </c>
-      <c r="Q8" s="2" t="s">
-        <v>37</v>
       </c>
       <c r="R8" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="S8" s="2" t="s">
+    </row>
+    <row r="9" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A9" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B9" s="2" t="s">
         <v>71</v>
       </c>
-    </row>
-    <row r="9" spans="1:19" x14ac:dyDescent="0.3">
-      <c r="A9" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="B9" s="2" t="s">
+      <c r="C9" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="C9" s="2" t="s">
+      <c r="D9" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="D9" s="2" t="s">
+      <c r="E9" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="F9" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="E9" s="2">
-        <v>8</v>
-      </c>
-      <c r="F9" s="2" t="s">
-        <v>23</v>
-      </c>
       <c r="G9" s="2" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="H9" s="2" t="s">
         <v>75</v>
       </c>
       <c r="I9" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="J9" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="K9" s="2">
+        <v>4</v>
+      </c>
+      <c r="L9" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="M9" s="2">
+        <v>40</v>
+      </c>
+      <c r="N9" s="2">
+        <v>60</v>
+      </c>
+      <c r="O9" s="2">
+        <v>100</v>
+      </c>
+      <c r="P9" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="Q9" s="2" t="s">
         <v>76</v>
-      </c>
-      <c r="J9" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="K9" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="L9" s="2">
-        <v>4</v>
-      </c>
-      <c r="M9" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="N9" s="2">
-        <v>40</v>
-      </c>
-      <c r="O9" s="2">
-        <v>60</v>
-      </c>
-      <c r="P9" s="2">
-        <v>100</v>
-      </c>
-      <c r="Q9" s="2" t="s">
-        <v>29</v>
       </c>
       <c r="R9" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="S9" s="2" t="s">
+    </row>
+    <row r="10" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A10" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="F10" s="2" t="s">
         <v>78</v>
       </c>
-    </row>
-    <row r="10" spans="1:19" x14ac:dyDescent="0.3">
-      <c r="A10" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>72</v>
-      </c>
-      <c r="C10" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="D10" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="E10" s="2">
-        <v>9</v>
-      </c>
-      <c r="F10" s="2" t="s">
-        <v>23</v>
-      </c>
       <c r="G10" s="2" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="H10" s="2" t="s">
         <v>79</v>
       </c>
       <c r="I10" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="J10" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="K10" s="2">
+        <v>5</v>
+      </c>
+      <c r="L10" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="M10" s="2">
+        <v>40</v>
+      </c>
+      <c r="N10" s="2">
+        <v>60</v>
+      </c>
+      <c r="O10" s="2">
+        <v>100</v>
+      </c>
+      <c r="P10" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="Q10" s="2" t="s">
         <v>80</v>
-      </c>
-      <c r="J10" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="K10" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="L10" s="2">
-        <v>5</v>
-      </c>
-      <c r="M10" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="N10" s="2">
-        <v>40</v>
-      </c>
-      <c r="O10" s="2">
-        <v>60</v>
-      </c>
-      <c r="P10" s="2">
-        <v>100</v>
-      </c>
-      <c r="Q10" s="2" t="s">
-        <v>37</v>
       </c>
       <c r="R10" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="S10" s="2" t="s">
+    </row>
+    <row r="11" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A11" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C11" s="2" t="s">
         <v>82</v>
       </c>
-    </row>
-    <row r="11" spans="1:19" x14ac:dyDescent="0.3">
-      <c r="A11" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="C11" s="2" t="s">
+      <c r="D11" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="D11" s="2" t="s">
+      <c r="E11" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="F11" s="2" t="s">
         <v>84</v>
-      </c>
-      <c r="E11" s="2">
-        <v>10</v>
-      </c>
-      <c r="F11" s="2" t="s">
-        <v>23</v>
       </c>
       <c r="G11" s="2" t="s">
         <v>85</v>
@@ -1368,57 +1334,54 @@
         <v>86</v>
       </c>
       <c r="I11" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="J11" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="K11" s="2">
+        <v>4</v>
+      </c>
+      <c r="L11" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="M11" s="2">
+        <v>35</v>
+      </c>
+      <c r="N11" s="2">
+        <v>65</v>
+      </c>
+      <c r="O11" s="2">
+        <v>100</v>
+      </c>
+      <c r="P11" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="Q11" s="2" t="s">
         <v>87</v>
-      </c>
-      <c r="J11" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="K11" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="L11" s="2">
-        <v>4</v>
-      </c>
-      <c r="M11" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="N11" s="2">
-        <v>35</v>
-      </c>
-      <c r="O11" s="2">
-        <v>65</v>
-      </c>
-      <c r="P11" s="2">
-        <v>100</v>
-      </c>
-      <c r="Q11" s="2" t="s">
-        <v>29</v>
       </c>
       <c r="R11" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="S11" s="2" t="s">
+    </row>
+    <row r="12" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A12" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="F12" s="2" t="s">
         <v>89</v>
-      </c>
-    </row>
-    <row r="12" spans="1:19" x14ac:dyDescent="0.3">
-      <c r="A12" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="B12" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>83</v>
-      </c>
-      <c r="D12" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="E12" s="2">
-        <v>11</v>
-      </c>
-      <c r="F12" s="2" t="s">
-        <v>23</v>
       </c>
       <c r="G12" s="2" t="s">
         <v>90</v>
@@ -1427,175 +1390,166 @@
         <v>91</v>
       </c>
       <c r="I12" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="J12" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="K12" s="2">
+        <v>4</v>
+      </c>
+      <c r="L12" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="M12" s="2">
+        <v>40</v>
+      </c>
+      <c r="N12" s="2">
+        <v>60</v>
+      </c>
+      <c r="O12" s="2">
+        <v>100</v>
+      </c>
+      <c r="P12" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="Q12" s="2" t="s">
         <v>92</v>
-      </c>
-      <c r="J12" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="K12" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="L12" s="2">
-        <v>4</v>
-      </c>
-      <c r="M12" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="N12" s="2">
-        <v>40</v>
-      </c>
-      <c r="O12" s="2">
-        <v>60</v>
-      </c>
-      <c r="P12" s="2">
-        <v>100</v>
-      </c>
-      <c r="Q12" s="2" t="s">
-        <v>37</v>
       </c>
       <c r="R12" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="S12" s="2" t="s">
+    </row>
+    <row r="13" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A13" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="B13" s="2" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="13" spans="1:19" x14ac:dyDescent="0.3">
-      <c r="A13" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="B13" s="2" t="s">
+      <c r="C13" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="D13" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="C13" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="D13" s="2" t="s">
+      <c r="E13" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="F13" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="E13" s="2">
-        <v>12</v>
-      </c>
-      <c r="F13" s="2" t="s">
-        <v>23</v>
-      </c>
       <c r="G13" s="2" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="H13" s="2" t="s">
         <v>97</v>
       </c>
       <c r="I13" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="J13" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="K13" s="2">
+        <v>4</v>
+      </c>
+      <c r="L13" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="M13" s="2">
+        <v>40</v>
+      </c>
+      <c r="N13" s="2">
+        <v>60</v>
+      </c>
+      <c r="O13" s="2">
+        <v>100</v>
+      </c>
+      <c r="P13" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="Q13" s="2" t="s">
         <v>98</v>
-      </c>
-      <c r="J13" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="K13" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="L13" s="2">
-        <v>4</v>
-      </c>
-      <c r="M13" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="N13" s="2">
-        <v>40</v>
-      </c>
-      <c r="O13" s="2">
-        <v>60</v>
-      </c>
-      <c r="P13" s="2">
-        <v>100</v>
-      </c>
-      <c r="Q13" s="2" t="s">
-        <v>29</v>
       </c>
       <c r="R13" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="S13" s="2" t="s">
+    </row>
+    <row r="14" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A14" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="F14" s="2" t="s">
         <v>100</v>
       </c>
-    </row>
-    <row r="14" spans="1:19" x14ac:dyDescent="0.3">
-      <c r="A14" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="B14" s="2" t="s">
-        <v>95</v>
-      </c>
-      <c r="C14" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="D14" s="2" t="s">
-        <v>96</v>
-      </c>
-      <c r="E14" s="2">
-        <v>13</v>
-      </c>
-      <c r="F14" s="2" t="s">
-        <v>23</v>
-      </c>
       <c r="G14" s="2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="H14" s="2" t="s">
         <v>101</v>
       </c>
       <c r="I14" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="J14" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="K14" s="2">
+        <v>4</v>
+      </c>
+      <c r="L14" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="M14" s="2">
+        <v>35</v>
+      </c>
+      <c r="N14" s="2">
+        <v>65</v>
+      </c>
+      <c r="O14" s="2">
+        <v>100</v>
+      </c>
+      <c r="P14" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="Q14" s="2" t="s">
         <v>102</v>
-      </c>
-      <c r="J14" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="K14" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="L14" s="2">
-        <v>4</v>
-      </c>
-      <c r="M14" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="N14" s="2">
-        <v>35</v>
-      </c>
-      <c r="O14" s="2">
-        <v>65</v>
-      </c>
-      <c r="P14" s="2">
-        <v>100</v>
-      </c>
-      <c r="Q14" s="2" t="s">
-        <v>37</v>
       </c>
       <c r="R14" s="2" t="s">
         <v>103</v>
       </c>
-      <c r="S14" s="2" t="s">
+    </row>
+    <row r="15" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A15" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C15" s="2" t="s">
         <v>104</v>
       </c>
-    </row>
-    <row r="15" spans="1:19" x14ac:dyDescent="0.3">
-      <c r="A15" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="B15" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="C15" s="2" t="s">
+      <c r="D15" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="D15" s="2" t="s">
+      <c r="E15" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="F15" s="2" t="s">
         <v>106</v>
-      </c>
-      <c r="E15" s="2">
-        <v>14</v>
-      </c>
-      <c r="F15" s="2" t="s">
-        <v>23</v>
       </c>
       <c r="G15" s="2" t="s">
         <v>107</v>
@@ -1604,57 +1558,54 @@
         <v>108</v>
       </c>
       <c r="I15" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="J15" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="K15" s="2">
+        <v>5</v>
+      </c>
+      <c r="L15" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="M15" s="2">
+        <v>40</v>
+      </c>
+      <c r="N15" s="2">
+        <v>60</v>
+      </c>
+      <c r="O15" s="2">
+        <v>100</v>
+      </c>
+      <c r="P15" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="Q15" s="2" t="s">
         <v>109</v>
-      </c>
-      <c r="J15" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="K15" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="L15" s="2">
-        <v>5</v>
-      </c>
-      <c r="M15" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="N15" s="2">
-        <v>40</v>
-      </c>
-      <c r="O15" s="2">
-        <v>60</v>
-      </c>
-      <c r="P15" s="2">
-        <v>100</v>
-      </c>
-      <c r="Q15" s="2" t="s">
-        <v>29</v>
       </c>
       <c r="R15" s="2" t="s">
         <v>110</v>
       </c>
-      <c r="S15" s="2" t="s">
+    </row>
+    <row r="16" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A16" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="E16" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="F16" s="2" t="s">
         <v>111</v>
-      </c>
-    </row>
-    <row r="16" spans="1:19" x14ac:dyDescent="0.3">
-      <c r="A16" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="B16" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="C16" s="2" t="s">
-        <v>105</v>
-      </c>
-      <c r="D16" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="E16" s="2">
-        <v>15</v>
-      </c>
-      <c r="F16" s="2" t="s">
-        <v>23</v>
       </c>
       <c r="G16" s="2" t="s">
         <v>112</v>
@@ -1663,37 +1614,34 @@
         <v>113</v>
       </c>
       <c r="I16" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="J16" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="K16" s="2">
+        <v>4</v>
+      </c>
+      <c r="L16" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="M16" s="2">
+        <v>30</v>
+      </c>
+      <c r="N16" s="2">
+        <v>70</v>
+      </c>
+      <c r="O16" s="2">
+        <v>100</v>
+      </c>
+      <c r="P16" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="Q16" s="2" t="s">
         <v>114</v>
-      </c>
-      <c r="J16" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="K16" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="L16" s="2">
-        <v>4</v>
-      </c>
-      <c r="M16" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="N16" s="2">
-        <v>30</v>
-      </c>
-      <c r="O16" s="2">
-        <v>70</v>
-      </c>
-      <c r="P16" s="2">
-        <v>100</v>
-      </c>
-      <c r="Q16" s="2" t="s">
-        <v>37</v>
       </c>
       <c r="R16" s="2" t="s">
         <v>115</v>
-      </c>
-      <c r="S16" s="2" t="s">
-        <v>116</v>
       </c>
     </row>
   </sheetData>

</xml_diff>